<commit_message>
ssid deseq; orthofinder; O2 flux
</commit_message>
<xml_diff>
--- a/tables/Table S3.xlsx
+++ b/tables/Table S3.xlsx
@@ -564,7 +564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J27"/>
+  <dimension ref="A1:J39"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="12.6640625" customWidth="1" style="17" min="1" max="1"/>
@@ -1312,7 +1312,7 @@
         </is>
       </c>
     </row>
-    <row r="22">
+    <row r="22" s="17">
       <c r="A22" s="18" t="inlineStr">
         <is>
           <t>Linear Mixed-Effects (Day-Averaged Calcification)</t>
@@ -1348,7 +1348,7 @@
         <v>0.046</v>
       </c>
     </row>
-    <row r="23">
+    <row r="23" s="17">
       <c r="B23" s="11" t="inlineStr">
         <is>
           <t>Site</t>
@@ -1381,7 +1381,7 @@
         <v>0.0065</v>
       </c>
     </row>
-    <row r="24">
+    <row r="24" s="17">
       <c r="B24" s="11" t="inlineStr">
         <is>
           <t>Site/Genotype</t>
@@ -1416,100 +1416,572 @@
         </is>
       </c>
     </row>
-    <row r="25">
+    <row r="25" s="17">
       <c r="A25" s="18" t="inlineStr">
         <is>
+          <t>Linear Mixed-Effects (Net Photosynthesis)</t>
+        </is>
+      </c>
+      <c r="B25" s="11" t="inlineStr">
+        <is>
+          <t>pH</t>
+        </is>
+      </c>
+      <c r="C25" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" s="9" t="n">
+        <v>3.6351</v>
+      </c>
+      <c r="E25" s="8" t="n">
+        <v>0.1158</v>
+      </c>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>0.086*</t>
+        </is>
+      </c>
+      <c r="G25" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H25" s="9" t="n">
+        <v>3.2872</v>
+      </c>
+      <c r="I25" s="8" t="n">
+        <v>0.0606</v>
+      </c>
+      <c r="J25" s="16" t="inlineStr">
+        <is>
+          <t>0.086*</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" s="17">
+      <c r="B26" s="11" t="inlineStr">
+        <is>
+          <t>Site</t>
+        </is>
+      </c>
+      <c r="C26" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="D26" s="9" t="n">
+        <v>0.3077</v>
+      </c>
+      <c r="E26" s="8" t="n">
+        <v>0.0396</v>
+      </c>
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>ns</t>
+        </is>
+      </c>
+      <c r="G26" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="H26" s="9" t="n">
+        <v>1.0588</v>
+      </c>
+      <c r="I26" s="8" t="n">
+        <v>0.1008</v>
+      </c>
+      <c r="J26" s="8" t="inlineStr">
+        <is>
+          <t>ns</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" s="17">
+      <c r="B27" s="11" t="inlineStr">
+        <is>
+          <t>Site/Genotype</t>
+        </is>
+      </c>
+      <c r="C27" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D27" s="9" t="n">
+        <v>0.2577</v>
+      </c>
+      <c r="E27" s="8" t="n">
+        <v>0.2832</v>
+      </c>
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>ns</t>
+        </is>
+      </c>
+      <c r="G27" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H27" s="9" t="n">
+        <v>0.6834</v>
+      </c>
+      <c r="I27" s="8" t="n">
+        <v>0.2648</v>
+      </c>
+      <c r="J27" s="8" t="inlineStr">
+        <is>
+          <t>ns</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" s="17">
+      <c r="A28" s="18" t="inlineStr">
+        <is>
+          <t>Linear Mixed-Effects (Respiration)</t>
+        </is>
+      </c>
+      <c r="B28" s="11" t="inlineStr">
+        <is>
+          <t>pH</t>
+        </is>
+      </c>
+      <c r="C28" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D28" s="9" t="n">
+        <v>0.2244</v>
+      </c>
+      <c r="E28" s="8" t="n">
+        <v>0.0027</v>
+      </c>
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>ns</t>
+        </is>
+      </c>
+      <c r="G28" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H28" s="9" t="n">
+        <v>1.0659</v>
+      </c>
+      <c r="I28" s="8" t="n">
+        <v>0.0204</v>
+      </c>
+      <c r="J28" s="16" t="inlineStr">
+        <is>
+          <t>ns</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" s="17">
+      <c r="B29" s="11" t="inlineStr">
+        <is>
+          <t>Site</t>
+        </is>
+      </c>
+      <c r="C29" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="D29" s="9" t="n">
+        <v>0.4411</v>
+      </c>
+      <c r="E29" s="8" t="n">
+        <v>0.0672</v>
+      </c>
+      <c r="F29" s="6" t="inlineStr">
+        <is>
+          <t>ns</t>
+        </is>
+      </c>
+      <c r="G29" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="H29" s="9" t="n">
+        <v>1.4174</v>
+      </c>
+      <c r="I29" s="8" t="n">
+        <v>0.1481</v>
+      </c>
+      <c r="J29" s="8" t="inlineStr">
+        <is>
+          <t>ns</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" s="17">
+      <c r="B30" s="11" t="inlineStr">
+        <is>
+          <t>Site/Genotype</t>
+        </is>
+      </c>
+      <c r="C30" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" s="8" t="n">
+        <v>0.3148</v>
+      </c>
+      <c r="F30" s="6" t="inlineStr">
+        <is>
+          <t>ns</t>
+        </is>
+      </c>
+      <c r="G30" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H30" s="9" t="n">
+        <v>1.0958</v>
+      </c>
+      <c r="I30" s="8" t="n">
+        <v>0.3363</v>
+      </c>
+      <c r="J30" s="8" t="inlineStr">
+        <is>
+          <t>ns</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" s="17">
+      <c r="A31" s="18" t="inlineStr">
+        <is>
+          <t>Linear Mixed-Effects (Gross Photosynthesis)</t>
+        </is>
+      </c>
+      <c r="B31" s="11" t="inlineStr">
+        <is>
+          <t>pH</t>
+        </is>
+      </c>
+      <c r="C31" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D31" s="9" t="n">
+        <v>1.574</v>
+      </c>
+      <c r="E31" s="8" t="n">
+        <v>0.024</v>
+      </c>
+      <c r="F31" s="6" t="inlineStr">
+        <is>
+          <t>ns</t>
+        </is>
+      </c>
+      <c r="G31" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H31" s="9" t="n">
+        <v>5.2864</v>
+      </c>
+      <c r="I31" s="8" t="n">
+        <v>0.08359999999999999</v>
+      </c>
+      <c r="J31" s="16" t="n">
+        <v>0.033</v>
+      </c>
+    </row>
+    <row r="32" s="17">
+      <c r="B32" s="11" t="inlineStr">
+        <is>
+          <t>Site</t>
+        </is>
+      </c>
+      <c r="C32" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="D32" s="9" t="n">
+        <v>0.4023</v>
+      </c>
+      <c r="E32" s="8" t="n">
+        <v>0.0682</v>
+      </c>
+      <c r="F32" s="6" t="inlineStr">
+        <is>
+          <t>ns</t>
+        </is>
+      </c>
+      <c r="G32" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="H32" s="9" t="n">
+        <v>0.7875</v>
+      </c>
+      <c r="I32" s="8" t="n">
+        <v>0.0868</v>
+      </c>
+      <c r="J32" s="8" t="inlineStr">
+        <is>
+          <t>ns</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" s="17">
+      <c r="B33" s="11" t="inlineStr">
+        <is>
+          <t>Site/Genotype</t>
+        </is>
+      </c>
+      <c r="C33" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D33" s="9" t="n">
+        <v>2.4509</v>
+      </c>
+      <c r="E33" s="8" t="n">
+        <v>0.781</v>
+      </c>
+      <c r="F33" s="6" t="inlineStr">
+        <is>
+          <t>ns</t>
+        </is>
+      </c>
+      <c r="G33" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H33" s="9" t="n">
+        <v>2.5534</v>
+      </c>
+      <c r="I33" s="8" t="n">
+        <v>0.4158</v>
+      </c>
+      <c r="J33" s="8" t="inlineStr">
+        <is>
+          <t>ns</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" s="17">
+      <c r="A34" s="18" t="inlineStr">
+        <is>
+          <t>Linear Mixed-Effects (Photosynthesis:Respiration)</t>
+        </is>
+      </c>
+      <c r="B34" s="11" t="inlineStr">
+        <is>
+          <t>pH</t>
+        </is>
+      </c>
+      <c r="C34" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D34" s="9" t="n">
+        <v>3.2377</v>
+      </c>
+      <c r="E34" s="8" t="n">
+        <v>0.1183</v>
+      </c>
+      <c r="F34" s="6" t="inlineStr">
+        <is>
+          <t>0.096*</t>
+        </is>
+      </c>
+      <c r="G34" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H34" s="9" t="n">
+        <v>6.5486</v>
+      </c>
+      <c r="I34" s="8" t="n">
+        <v>0.1469</v>
+      </c>
+      <c r="J34" s="16" t="n">
+        <v>0.019</v>
+      </c>
+    </row>
+    <row r="35" s="17">
+      <c r="B35" s="11" t="inlineStr">
+        <is>
+          <t>Site</t>
+        </is>
+      </c>
+      <c r="C35" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="D35" s="9" t="n">
+        <v>0.3918</v>
+      </c>
+      <c r="E35" s="8" t="n">
+        <v>0.051</v>
+      </c>
+      <c r="F35" s="6" t="inlineStr">
+        <is>
+          <t>ns</t>
+        </is>
+      </c>
+      <c r="G35" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="H35" s="9" t="n">
+        <v>1.749</v>
+      </c>
+      <c r="I35" s="8" t="n">
+        <v>0.129</v>
+      </c>
+      <c r="J35" s="8" t="inlineStr">
+        <is>
+          <t>ns</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" s="17">
+      <c r="B36" s="11" t="inlineStr">
+        <is>
+          <t>Site/Genotype</t>
+        </is>
+      </c>
+      <c r="C36" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D36" s="9" t="n">
+        <v>0.0179</v>
+      </c>
+      <c r="E36" s="8" t="n">
+        <v>0.1303</v>
+      </c>
+      <c r="F36" s="6" t="inlineStr">
+        <is>
+          <t>ns</t>
+        </is>
+      </c>
+      <c r="G36" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H36" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I36" s="8" t="n">
+        <v>0.06279999999999999</v>
+      </c>
+      <c r="J36" s="8" t="inlineStr">
+        <is>
+          <t>ns</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="18" t="inlineStr">
+        <is>
           <t>PERMANOVA (Transcriptomics)</t>
         </is>
       </c>
-      <c r="B25" s="11" t="inlineStr">
+      <c r="B37" s="11" t="inlineStr">
         <is>
           <t>Colony (genotype)</t>
         </is>
       </c>
-      <c r="C25" s="14" t="n">
+      <c r="C37" s="14" t="n">
         <v>20</v>
       </c>
-      <c r="D25" s="15" t="inlineStr">
+      <c r="D37" s="15" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="E25" s="14" t="n">
-        <v>0.642</v>
-      </c>
-      <c r="F25" s="11" t="inlineStr">
+      <c r="E37" s="14" t="n">
+        <v>0.641</v>
+      </c>
+      <c r="F37" s="11" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="G25" s="14" t="n"/>
-      <c r="H25" s="14" t="n"/>
-      <c r="I25" s="14" t="n"/>
-      <c r="J25" s="14" t="n"/>
-    </row>
-    <row r="26">
-      <c r="B26" s="11" t="inlineStr">
+      <c r="G37" s="14" t="n">
+        <v>19</v>
+      </c>
+      <c r="H37" s="15" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I37" s="14" t="n">
+        <v>0.467</v>
+      </c>
+      <c r="J37" s="11" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="11" t="inlineStr">
         <is>
           <t>Treatment (within colony)</t>
         </is>
       </c>
-      <c r="C26" s="14" t="n">
-        <v>3</v>
-      </c>
-      <c r="D26" s="15" t="n">
+      <c r="C38" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="D38" s="15" t="n">
         <v>2.3162</v>
       </c>
-      <c r="E26" s="14" t="n">
+      <c r="E38" s="14" t="n">
         <v>0.076</v>
       </c>
-      <c r="F26" s="11" t="inlineStr">
+      <c r="F38" s="11" t="inlineStr">
         <is>
           <t>&lt;0.001</t>
         </is>
       </c>
-      <c r="G26" s="14" t="n"/>
-      <c r="H26" s="14" t="n"/>
-      <c r="I26" s="14" t="n"/>
-      <c r="J26" s="14" t="n"/>
-    </row>
-    <row r="27">
-      <c r="B27" s="11" t="inlineStr">
+      <c r="G38" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="H38" s="15" t="n">
+        <v>2.7452</v>
+      </c>
+      <c r="I38" s="14" t="n">
+        <v>0.07099999999999999</v>
+      </c>
+      <c r="J38" s="11" t="inlineStr">
+        <is>
+          <t>&lt;0.001</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="11" t="inlineStr">
         <is>
           <t>Urban vs Reef (colony means)</t>
         </is>
       </c>
-      <c r="C27" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="D27" s="15" t="n">
+      <c r="C39" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D39" s="15" t="n">
         <v>1.4387</v>
       </c>
-      <c r="E27" s="14" t="n">
+      <c r="E39" s="14" t="n">
         <v>0.07000000000000001</v>
       </c>
-      <c r="F27" s="11" t="inlineStr">
+      <c r="F39" s="11" t="inlineStr">
         <is>
           <t>0.094*</t>
         </is>
       </c>
-      <c r="G27" s="14" t="n"/>
-      <c r="H27" s="14" t="n"/>
-      <c r="I27" s="14" t="n"/>
-      <c r="J27" s="14" t="n"/>
+      <c r="G39" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="H39" s="15" t="n">
+        <v>1.1302</v>
+      </c>
+      <c r="I39" s="14" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="J39" s="11" t="inlineStr">
+        <is>
+          <t>ns</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="16">
     <mergeCell ref="A8:A10"/>
     <mergeCell ref="A16:A18"/>
+    <mergeCell ref="A34:A36"/>
     <mergeCell ref="A3:A4"/>
     <mergeCell ref="A25:A27"/>
+    <mergeCell ref="A28:A30"/>
+    <mergeCell ref="A31:A33"/>
     <mergeCell ref="A19:A21"/>
     <mergeCell ref="A5:A7"/>
     <mergeCell ref="B1:B2"/>
     <mergeCell ref="G1:J1"/>
     <mergeCell ref="C1:F1"/>
     <mergeCell ref="A11:A15"/>
+    <mergeCell ref="A37:A39"/>
     <mergeCell ref="A22:A24"/>
     <mergeCell ref="A1:A2"/>
   </mergeCells>

</xml_diff>

<commit_message>
differential expression with dream
</commit_message>
<xml_diff>
--- a/tables/Table S3.xlsx
+++ b/tables/Table S3.xlsx
@@ -564,7 +564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J39"/>
+  <dimension ref="A1:J40"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="12.6640625" customWidth="1" style="17" min="1" max="1"/>
@@ -1896,7 +1896,7 @@
         </is>
       </c>
     </row>
-    <row r="38">
+    <row r="38" s="17">
       <c r="B38" s="11" t="inlineStr">
         <is>
           <t>Treatment (within colony)</t>
@@ -1931,36 +1931,71 @@
         </is>
       </c>
     </row>
-    <row r="39">
+    <row r="39" s="17">
       <c r="B39" s="11" t="inlineStr">
         <is>
+          <t>Site (colony means)</t>
+        </is>
+      </c>
+      <c r="C39" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="D39" s="15" t="n">
+        <v>1.1536</v>
+      </c>
+      <c r="E39" s="14" t="n">
+        <v>0.169</v>
+      </c>
+      <c r="F39" s="11" t="inlineStr">
+        <is>
+          <t>ns</t>
+        </is>
+      </c>
+      <c r="G39" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="H39" s="15" t="n">
+        <v>0.9865</v>
+      </c>
+      <c r="I39" s="14" t="n">
+        <v>0.156</v>
+      </c>
+      <c r="J39" s="11" t="inlineStr">
+        <is>
+          <t>ns</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="11" t="inlineStr">
+        <is>
           <t>Urban vs Reef (colony means)</t>
         </is>
       </c>
-      <c r="C39" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="D39" s="15" t="n">
+      <c r="C40" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D40" s="15" t="n">
         <v>1.4387</v>
       </c>
-      <c r="E39" s="14" t="n">
+      <c r="E40" s="14" t="n">
         <v>0.07000000000000001</v>
       </c>
-      <c r="F39" s="11" t="inlineStr">
+      <c r="F40" s="11" t="inlineStr">
         <is>
           <t>0.094*</t>
         </is>
       </c>
-      <c r="G39" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="H39" s="15" t="n">
+      <c r="G40" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="H40" s="15" t="n">
         <v>1.1302</v>
       </c>
-      <c r="I39" s="14" t="n">
+      <c r="I40" s="14" t="n">
         <v>0.059</v>
       </c>
-      <c r="J39" s="11" t="inlineStr">
+      <c r="J40" s="11" t="inlineStr">
         <is>
           <t>ns</t>
         </is>
@@ -1974,14 +2009,14 @@
     <mergeCell ref="A3:A4"/>
     <mergeCell ref="A25:A27"/>
     <mergeCell ref="A28:A30"/>
-    <mergeCell ref="A31:A33"/>
     <mergeCell ref="A19:A21"/>
     <mergeCell ref="A5:A7"/>
     <mergeCell ref="B1:B2"/>
     <mergeCell ref="G1:J1"/>
     <mergeCell ref="C1:F1"/>
+    <mergeCell ref="A31:A33"/>
     <mergeCell ref="A11:A15"/>
-    <mergeCell ref="A37:A39"/>
+    <mergeCell ref="A37:A40"/>
     <mergeCell ref="A22:A24"/>
     <mergeCell ref="A1:A2"/>
   </mergeCells>

</xml_diff>